<commit_message>
Add Expenses and Revenue sheets to normal_multi_sheet.xlsx
Adds 12 expense transactions and 15 revenue transactions using products
and suppliers/customers already present in the file. All columns match
the expected import schema (ID, Date, Supplier/Customer ID, Product,
Unit Price, Tax, Total, Reference, Payment Method/Status, Shipping).

https://claude.ai/code/session_01Dk89YSzD4ocarUwTp71Pc8
</commit_message>
<xml_diff>
--- a/TestData/normal_multi_sheet.xlsx
+++ b/TestData/normal_multi_sheet.xlsx
@@ -10,6 +10,8 @@
     <sheet name="Customers" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Products" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Suppliers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Expenses" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Revenue" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -48,8 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -666,7 +671,6 @@
           <t>US</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>Active</t>
@@ -792,7 +796,6 @@
           <t>US</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>Active</t>
@@ -1113,7 +1116,6 @@
           <t>US</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
           <t>Active</t>
@@ -1304,7 +1306,6 @@
           <t>US</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>Active</t>
@@ -1781,7 +1782,6 @@
           <t>End-of-quarter business tax preparation</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>Adams &amp; Associates</t>
@@ -1825,7 +1825,6 @@
           <t>Full-service monthly bookkeeping</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Foster Accounting</t>
@@ -2626,4 +2625,1270 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Supplier ID</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Unit Price</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Tax</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Payment Method</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Shipping</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PUR-001</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>45672</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SUP-001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Industrial Drill Press</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>899.99</v>
+      </c>
+      <c r="F2" t="n">
+        <v>72</v>
+      </c>
+      <c r="G2" t="n">
+        <v>971.99</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>INV-MW-4401</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>BankTransfer</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PUR-002</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>45679</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SUP-002</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Premium Wood Stain - Oak</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>189</v>
+      </c>
+      <c r="F3" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="G3" t="n">
+        <v>204.12</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>INV-SW-7720</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>CreditCard</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PUR-003</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>45691</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>SUP-004</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Copper Pipe 3/4" x 10ft</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>450</v>
+      </c>
+      <c r="F4" t="n">
+        <v>36</v>
+      </c>
+      <c r="G4" t="n">
+        <v>486</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>INV-NP-3310</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>BankTransfer</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PUR-004</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>45698</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SUP-005</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Safety Goggles Anti-Fog</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>250</v>
+      </c>
+      <c r="F5" t="n">
+        <v>20</v>
+      </c>
+      <c r="G5" t="n">
+        <v>270</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>INV-3M-5500</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>CreditCard</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PUR-005</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>45706</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SUP-006</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Quarterly Tax Filing</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1200</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>INV-AA-0901</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PUR-006</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>45717</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SUP-003</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>LED Panel Light 2x4</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>640</v>
+      </c>
+      <c r="F7" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="G7" t="n">
+        <v>691.2</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>INV-BS-2200</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>BankTransfer</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PUR-007</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>45728</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SUP-008</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Concrete Mix 80lb Bag</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>375</v>
+      </c>
+      <c r="F8" t="n">
+        <v>30</v>
+      </c>
+      <c r="G8" t="n">
+        <v>405</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>INV-QK-1100</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>DebitCard</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PUR-008</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>45741</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SUP-007</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Monthly Bookkeeping</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>500</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>500</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>INV-FA-0302</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>BankTransfer</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PUR-009</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>45752</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>SUP-009</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Electrical Wire 12AWG 250ft</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>330</v>
+      </c>
+      <c r="F10" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="G10" t="n">
+        <v>356.4</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>INV-NW-6600</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>CreditCard</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PUR-010</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>45761</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SUP-001</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Pressure Washer 3000PSI</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>749</v>
+      </c>
+      <c r="F11" t="n">
+        <v>59.92</v>
+      </c>
+      <c r="G11" t="n">
+        <v>808.92</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>INV-MW-4402</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>BankTransfer</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PUR-011</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>45775</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>SUP-010</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Equipment Rental - Excavator</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>2200</v>
+      </c>
+      <c r="F12" t="n">
+        <v>176</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2376</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>INV-UR-8800</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>BankTransfer</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PUR-012</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>45783</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SUP-002</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Premium Wood Stain - Oak</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>378</v>
+      </c>
+      <c r="F13" t="n">
+        <v>30.24</v>
+      </c>
+      <c r="G13" t="n">
+        <v>408.24</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>INV-SW-7721</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>CreditCard</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Customer ID</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Unit Price</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Tax</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Payment Status</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Shipping</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SAL-001</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>45667</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CUST-004</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Industrial Drill Press</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1299.99</v>
+      </c>
+      <c r="F2" t="n">
+        <v>104</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1403.99</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>SO-10001</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SAL-002</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>45675</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CUST-001</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Premium Wood Stain - Oak</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>349</v>
+      </c>
+      <c r="F3" t="n">
+        <v>27.92</v>
+      </c>
+      <c r="G3" t="n">
+        <v>376.92</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>SO-10002</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SAL-003</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>45687</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CUST-006</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>LED Panel Light 2x4</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>960</v>
+      </c>
+      <c r="F4" t="n">
+        <v>76.8</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1036.8</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>SO-10003</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SAL-004</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>45696</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CUST-009</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Copper Pipe 3/4" x 10ft</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>780</v>
+      </c>
+      <c r="F5" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="G5" t="n">
+        <v>842.4</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>SO-10004</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SAL-005</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>45702</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CUST-002</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Safety Goggles Anti-Fog</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>499.5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>39.96</v>
+      </c>
+      <c r="G6" t="n">
+        <v>539.46</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>SO-10005</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SAL-006</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>45713</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CUST-011</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Pressure Washer 3000PSI</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1149</v>
+      </c>
+      <c r="F7" t="n">
+        <v>91.92</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1240.92</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>SO-10006</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SAL-007</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>45721</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CUST-003</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Concrete Mix 80lb Bag</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>562.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>45</v>
+      </c>
+      <c r="G8" t="n">
+        <v>607.5</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>SO-10007</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SAL-008</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>45731</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CUST-014</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Electrical Wire 12AWG 250ft</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>495</v>
+      </c>
+      <c r="F9" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="G9" t="n">
+        <v>534.6</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>SO-10008</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SAL-009</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>45744</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CUST-007</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>LED Panel Light 2x4</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>480</v>
+      </c>
+      <c r="F10" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="G10" t="n">
+        <v>518.4</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>SO-10009</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SAL-010</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>45749</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CUST-012</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Industrial Drill Press</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1299.99</v>
+      </c>
+      <c r="F11" t="n">
+        <v>104</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1403.99</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>SO-10010</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SAL-011</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>45765</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CUST-005</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Premium Wood Stain - Oak</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>174.5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>13.96</v>
+      </c>
+      <c r="G12" t="n">
+        <v>188.46</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>SO-10011</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SAL-012</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>45777</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CUST-008</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Copper Pipe 3/4" x 10ft</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>520</v>
+      </c>
+      <c r="F13" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="G13" t="n">
+        <v>561.6</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>SO-10012</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SAL-013</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>45787</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CUST-010</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Safety Goggles Anti-Fog</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>332.5</v>
+      </c>
+      <c r="F14" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="G14" t="n">
+        <v>359.1</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>SO-10013</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SAL-014</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>45797</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CUST-013</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Concrete Mix 80lb Bag</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>375</v>
+      </c>
+      <c r="F15" t="n">
+        <v>30</v>
+      </c>
+      <c r="G15" t="n">
+        <v>405</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>SO-10014</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SAL-015</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="n">
+        <v>45805</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CUST-004</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Pressure Washer 3000PSI</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1149</v>
+      </c>
+      <c r="F16" t="n">
+        <v>91.92</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1240.92</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>SO-10015</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>